<commit_message>
add codfe for diag runs
Ref: None
</commit_message>
<xml_diff>
--- a/angle_calculator.xlsx
+++ b/angle_calculator.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>ширина робота</t>
   </si>
@@ -34,6 +34,9 @@
   </si>
   <si>
     <t>длина внутренней дуги</t>
+  </si>
+  <si>
+    <t>диагональ</t>
   </si>
 </sst>
 </file>
@@ -372,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="15.140625" bestFit="1" customWidth="1"/>
@@ -455,6 +458,109 @@
         <v>0.40625</v>
       </c>
     </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <f>$A$2 + $B$2/2</f>
+        <v>218</v>
+      </c>
+      <c r="D8">
+        <f>$A$2 - $B$2/2</f>
+        <v>142</v>
+      </c>
+      <c r="E8">
+        <v>400</v>
+      </c>
+      <c r="F8">
+        <f>$D$8 * E8 /$C$8</f>
+        <v>260.55045871559633</v>
+      </c>
+      <c r="G8">
+        <f>F8/E8</f>
+        <v>0.65137614678899081</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E9">
+        <v>600</v>
+      </c>
+      <c r="F9">
+        <f>$D$2 * E9 /$C$2</f>
+        <v>243.75</v>
+      </c>
+      <c r="G9">
+        <f>F9/E9</f>
+        <v>0.40625</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E10">
+        <v>700</v>
+      </c>
+      <c r="F10">
+        <f>$D$2 * E10 /$C$2</f>
+        <v>284.375</v>
+      </c>
+      <c r="G10">
+        <f>F10/E10</f>
+        <v>0.40625</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <f>SQRT(2 *A2/2 *A2/2)</f>
+        <v>127.27922061357856</v>
+      </c>
+      <c r="C13">
+        <f>$A$13 + $B$2/2</f>
+        <v>165.27922061357856</v>
+      </c>
+      <c r="D13">
+        <f>$A$13 - $B$2/2</f>
+        <v>89.279220613578559</v>
+      </c>
+      <c r="E13">
+        <v>400</v>
+      </c>
+      <c r="F13">
+        <f>$D$8 * E13 /$C$8</f>
+        <v>260.55045871559633</v>
+      </c>
+      <c r="G13">
+        <f>F13/E13</f>
+        <v>0.65137614678899081</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E14">
+        <v>600</v>
+      </c>
+      <c r="F14">
+        <f>$D$2 * E14 /$C$2</f>
+        <v>243.75</v>
+      </c>
+      <c r="G14">
+        <f>F14/E14</f>
+        <v>0.40625</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E15">
+        <v>700</v>
+      </c>
+      <c r="F15">
+        <f>$D$2 * E15 /$C$2</f>
+        <v>284.375</v>
+      </c>
+      <c r="G15">
+        <f>F15/E15</f>
+        <v>0.40625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>